<commit_message>
Análisis semanal: cola y reportes
</commit_message>
<xml_diff>
--- a/reportes/cults3d_mercado.xlsx
+++ b/reportes/cults3d_mercado.xlsx
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>126034</v>
+        <v>126035</v>
       </c>
     </row>
     <row r="5">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1862282.66</v>
+        <v>1862293.89</v>
       </c>
     </row>
     <row r="6">
@@ -886,7 +886,7 @@
         <v>254205</v>
       </c>
       <c r="H7" t="n">
-        <v>0.265661252900232</v>
+        <v>0.2656415694591728</v>
       </c>
       <c r="I7" t="n">
         <v>1</v>
@@ -932,7 +932,7 @@
         <v>224260</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2656415694591728</v>
+        <v>0.2653534183082271</v>
       </c>
       <c r="I8" t="n">
         <v>1</v>
@@ -978,7 +978,7 @@
         <v>224260</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2656415694591728</v>
+        <v>0.2653534183082271</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
@@ -1024,7 +1024,7 @@
         <v>224260</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2656415694591728</v>
+        <v>0.2653534183082271</v>
       </c>
       <c r="I10" t="n">
         <v>1</v>
@@ -1070,7 +1070,7 @@
         <v>243665</v>
       </c>
       <c r="H11" t="n">
-        <v>0.266235973466049</v>
+        <v>0.2662261317455195</v>
       </c>
       <c r="I11" t="n">
         <v>1</v>
@@ -1162,7 +1162,7 @@
         <v>319315.3</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2656514111797024</v>
+        <v>0.2654974938837</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
@@ -1254,7 +1254,7 @@
         <v>254205</v>
       </c>
       <c r="H15" t="n">
-        <v>0.265661252900232</v>
+        <v>0.2656415694591728</v>
       </c>
       <c r="I15" t="n">
         <v>1</v>
@@ -1668,7 +1668,7 @@
         <v>255407.58</v>
       </c>
       <c r="H24" t="n">
-        <v>0.2637475088675174</v>
+        <v>0.2636034332920446</v>
       </c>
       <c r="I24" t="n">
         <v>1</v>
@@ -1806,7 +1806,7 @@
         <v>440715</v>
       </c>
       <c r="H27" t="n">
-        <v>0.3086522462562396</v>
+        <v>0.3083604777415853</v>
       </c>
       <c r="I27" t="n">
         <v>1</v>
@@ -3367,7 +3367,7 @@
         <v>3.96</v>
       </c>
       <c r="G61" t="n">
-        <v>31586.68</v>
+        <v>31597.91</v>
       </c>
       <c r="H61" t="n">
         <v>0.03709285622964752</v>
@@ -3600,7 +3600,7 @@
         <v>281235</v>
       </c>
       <c r="H66" t="n">
-        <v>0.265661252900232</v>
+        <v>0.2656415694591728</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
@@ -4488,7 +4488,7 @@
         <v>11.23</v>
       </c>
       <c r="F4" t="n">
-        <v>48039.85</v>
+        <v>48051.08</v>
       </c>
       <c r="G4" t="n">
         <v>0.0267175572519084</v>
@@ -4644,7 +4644,7 @@
         <v>11.23</v>
       </c>
       <c r="F2" t="n">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="G2" t="n">
         <v>177</v>
@@ -4664,13 +4664,13 @@
         <v>7</v>
       </c>
       <c r="L2" t="n">
-        <v>60.28571428571428</v>
+        <v>60.35714285714285</v>
       </c>
       <c r="M2" t="n">
-        <v>9478.120000000001</v>
+        <v>9489.35</v>
       </c>
       <c r="N2" t="n">
-        <v>0.03303973380309258</v>
+        <v>0.03307888040712468</v>
       </c>
       <c r="O2" t="b">
         <v>0</v>
@@ -5494,12 +5494,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Frieren Bust 3D Print</t>
+          <t>Claire Bust 3D Print</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:5020434</t>
+          <t>https://cults3d.com/:5020453</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5508,7 +5508,7 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46301.76526620371</v>
+        <v>46301.76777777778</v>
       </c>
       <c r="E17" t="n">
         <v>15</v>
@@ -5517,17 +5517,17 @@
         <v>417</v>
       </c>
       <c r="G17" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H17" t="n">
-        <v>980</v>
+        <v>783</v>
       </c>
       <c r="I17" t="b">
         <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3dprint, anime, fanart, fantasy, figurine, frieren, mage, stl</t>
+          <t>claire, evil, female, figure, handgun, jacket, re, redfield, resident, survivor, veronica</t>
         </is>
       </c>
       <c r="K17" t="n">
@@ -5540,7 +5540,7 @@
         <v>6255</v>
       </c>
       <c r="N17" t="n">
-        <v>0.4255102040816326</v>
+        <v>0.5325670498084292</v>
       </c>
       <c r="O17" t="b">
         <v>0</v>
@@ -5552,12 +5552,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Claire Bust 3D Print</t>
+          <t>Frieren Bust 3D Print</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:5020453</t>
+          <t>https://cults3d.com/:5020434</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5566,7 +5566,7 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46301.76777777778</v>
+        <v>46301.76526620371</v>
       </c>
       <c r="E18" t="n">
         <v>15</v>
@@ -5575,17 +5575,17 @@
         <v>417</v>
       </c>
       <c r="G18" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H18" t="n">
-        <v>783</v>
+        <v>980</v>
       </c>
       <c r="I18" t="b">
         <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>claire, evil, female, figure, handgun, jacket, re, redfield, resident, survivor, veronica</t>
+          <t>3dprint, anime, fanart, fantasy, figurine, frieren, mage, stl</t>
         </is>
       </c>
       <c r="K18" t="n">
@@ -5598,7 +5598,7 @@
         <v>6255</v>
       </c>
       <c r="N18" t="n">
-        <v>0.5325670498084292</v>
+        <v>0.4255102040816326</v>
       </c>
       <c r="O18" t="b">
         <v>0</v>
@@ -5842,12 +5842,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Anakin Ronin Bust 3D Print</t>
+          <t>Shanoa Bust 3D Print</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:5021462</t>
+          <t>https://cults3d.com/:5020467</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="D23" s="1" t="n">
-        <v>46301.93331018519</v>
+        <v>46301.77025462963</v>
       </c>
       <c r="E23" t="n">
         <v>15</v>
@@ -5865,17 +5865,17 @@
         <v>412</v>
       </c>
       <c r="G23" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H23" t="n">
-        <v>1256</v>
+        <v>753</v>
       </c>
       <c r="I23" t="b">
         <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>ahsoka, anakin, clone, darth, jedi, lightsaber, maul, rebels, sith, star, stormtrooper, tano, vader, wars</t>
+          <t>boss, castlevania, dracul, dracula, king, shanoa, vampire</t>
         </is>
       </c>
       <c r="K23" t="n">
@@ -5888,10 +5888,10 @@
         <v>6180</v>
       </c>
       <c r="N23" t="n">
-        <v>0.3280254777070064</v>
+        <v>0.547144754316069</v>
       </c>
       <c r="O23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" t="b">
         <v>0</v>
@@ -5900,12 +5900,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Shanoa Bust 3D Print</t>
+          <t>Anakin Ronin Bust 3D Print</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:5020467</t>
+          <t>https://cults3d.com/:5021462</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -5914,7 +5914,7 @@
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>46301.77025462963</v>
+        <v>46301.93331018519</v>
       </c>
       <c r="E24" t="n">
         <v>15</v>
@@ -5923,17 +5923,17 @@
         <v>412</v>
       </c>
       <c r="G24" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H24" t="n">
-        <v>753</v>
+        <v>1256</v>
       </c>
       <c r="I24" t="b">
         <v>0</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>boss, castlevania, dracul, dracula, king, shanoa, vampire</t>
+          <t>ahsoka, anakin, clone, darth, jedi, lightsaber, maul, rebels, sith, star, stormtrooper, tano, vader, wars</t>
         </is>
       </c>
       <c r="K24" t="n">
@@ -5946,10 +5946,10 @@
         <v>6180</v>
       </c>
       <c r="N24" t="n">
-        <v>0.547144754316069</v>
+        <v>0.3280254777070064</v>
       </c>
       <c r="O24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" t="b">
         <v>0</v>
@@ -6158,7 +6158,7 @@
         <v>19</v>
       </c>
       <c r="H28" t="n">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="I28" t="b">
         <v>0</v>
@@ -6178,7 +6178,7 @@
         <v>5680</v>
       </c>
       <c r="N28" t="n">
-        <v>0.308695652173913</v>
+        <v>0.3083604777415853</v>
       </c>
       <c r="O28" t="b">
         <v>1</v>
@@ -6912,7 +6912,7 @@
         <v>18</v>
       </c>
       <c r="H41" t="n">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
@@ -6932,7 +6932,7 @@
         <v>4580</v>
       </c>
       <c r="N41" t="n">
-        <v>0.265661252900232</v>
+        <v>0.2653534183082271</v>
       </c>
       <c r="O41" t="b">
         <v>0</v>
@@ -8104,12 +8104,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Savage Land Psylocke Bust 3D Print</t>
+          <t>Cowgirl Rogue Bust 3D Print</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:4878923</t>
+          <t>https://cults3d.com/:4878931</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -8118,7 +8118,7 @@
         </is>
       </c>
       <c r="D62" s="1" t="n">
-        <v>46271.73194444444</v>
+        <v>46271.73293981481</v>
       </c>
       <c r="E62" t="n">
         <v>15</v>
@@ -8127,17 +8127,17 @@
         <v>679</v>
       </c>
       <c r="G62" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H62" t="n">
-        <v>1831</v>
+        <v>1790</v>
       </c>
       <c r="I62" t="b">
         <v>0</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>art, comics, fan, female, figure, figurine, game, garage, kit, miniature, miniatures, movie, psylocke, savage, sculpture, stylized, tabletop, video, xmen</t>
+          <t>cosplay, costume, cowboy, cowgirl, marvel, parts, rebel, rivals, rogue, starlit</t>
         </is>
       </c>
       <c r="K62" t="n">
@@ -8150,7 +8150,7 @@
         <v>10185</v>
       </c>
       <c r="N62" t="n">
-        <v>0.3708356089568542</v>
+        <v>0.3793296089385475</v>
       </c>
       <c r="O62" t="b">
         <v>1</v>
@@ -8162,12 +8162,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Cowgirl Rogue Bust 3D Print</t>
+          <t>Savage Land Psylocke Bust 3D Print</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:4878931</t>
+          <t>https://cults3d.com/:4878923</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -8176,7 +8176,7 @@
         </is>
       </c>
       <c r="D63" s="1" t="n">
-        <v>46271.73293981481</v>
+        <v>46271.73194444444</v>
       </c>
       <c r="E63" t="n">
         <v>15</v>
@@ -8185,17 +8185,17 @@
         <v>679</v>
       </c>
       <c r="G63" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H63" t="n">
-        <v>1790</v>
+        <v>1831</v>
       </c>
       <c r="I63" t="b">
         <v>0</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>cosplay, costume, cowboy, cowgirl, marvel, parts, rebel, rivals, rogue, starlit</t>
+          <t>art, comics, fan, female, figure, figurine, game, garage, kit, miniature, miniatures, movie, psylocke, savage, sculpture, stylized, tabletop, video, xmen</t>
         </is>
       </c>
       <c r="K63" t="n">
@@ -8208,7 +8208,7 @@
         <v>10185</v>
       </c>
       <c r="N63" t="n">
-        <v>0.3793296089385475</v>
+        <v>0.3708356089568542</v>
       </c>
       <c r="O63" t="b">
         <v>1</v>
@@ -8478,7 +8478,7 @@
         <v>22</v>
       </c>
       <c r="H68" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="I68" t="b">
         <v>0</v>
@@ -8498,7 +8498,7 @@
         <v>3980</v>
       </c>
       <c r="N68" t="n">
-        <v>0.3080495356037152</v>
+        <v>0.3075734157650695</v>
       </c>
       <c r="O68" t="b">
         <v>1</v>
@@ -8536,7 +8536,7 @@
         <v>18</v>
       </c>
       <c r="H69" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="I69" t="b">
         <v>0</v>
@@ -8556,7 +8556,7 @@
         <v>3980</v>
       </c>
       <c r="N69" t="n">
-        <v>0.3114241001564945</v>
+        <v>0.3109375</v>
       </c>
       <c r="O69" t="b">
         <v>1</v>
@@ -9844,12 +9844,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Big Daddy and Little Sister - BioShock - Bust</t>
+          <t>Deku - My Hero Academia - Bust</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:4971763</t>
+          <t>https://cults3d.com/:4971767</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -9858,7 +9858,7 @@
         </is>
       </c>
       <c r="D92" s="1" t="n">
-        <v>46292.21859953704</v>
+        <v>46292.21883101852</v>
       </c>
       <c r="E92" t="n">
         <v>13.49</v>
@@ -9867,17 +9867,17 @@
         <v>306</v>
       </c>
       <c r="G92" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H92" t="n">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="I92" t="b">
         <v>0</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>big daddy, bioshock, bust, fanart, miniature, resin, stl</t>
+          <t>bust, deku, fanart, miniature, my hero academia, resin, stl</t>
         </is>
       </c>
       <c r="K92" t="n">
@@ -9890,7 +9890,7 @@
         <v>4127.940000000001</v>
       </c>
       <c r="N92" t="n">
-        <v>0.6035502958579881</v>
+        <v>0.6144578313253012</v>
       </c>
       <c r="O92" t="b">
         <v>0</v>
@@ -9902,12 +9902,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Deku - My Hero Academia - Bust</t>
+          <t>Big Daddy and Little Sister - BioShock - Bust</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:4971767</t>
+          <t>https://cults3d.com/:4971763</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -9916,7 +9916,7 @@
         </is>
       </c>
       <c r="D93" s="1" t="n">
-        <v>46292.21883101852</v>
+        <v>46292.21859953704</v>
       </c>
       <c r="E93" t="n">
         <v>13.49</v>
@@ -9925,17 +9925,17 @@
         <v>306</v>
       </c>
       <c r="G93" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H93" t="n">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="I93" t="b">
         <v>0</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>bust, deku, fanart, miniature, my hero academia, resin, stl</t>
+          <t>big daddy, bioshock, bust, fanart, miniature, resin, stl</t>
         </is>
       </c>
       <c r="K93" t="n">
@@ -9948,7 +9948,7 @@
         <v>4127.940000000001</v>
       </c>
       <c r="N93" t="n">
-        <v>0.6144578313253012</v>
+        <v>0.6035502958579881</v>
       </c>
       <c r="O93" t="b">
         <v>0</v>
@@ -10018,12 +10018,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Proxima the Broodseeker</t>
+          <t>pin head Fan art (no ams-multiparts/3mf)</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:5079132</t>
+          <t>https://cults3d.com/:5055346</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -10032,42 +10032,42 @@
         </is>
       </c>
       <c r="D95" s="1" t="n">
-        <v>46313.49111111111</v>
+        <v>46308.81805555556</v>
       </c>
       <c r="E95" t="n">
-        <v>17.6</v>
+        <v>3.96</v>
       </c>
       <c r="F95" t="n">
         <v>158</v>
       </c>
       <c r="G95" t="n">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="H95" t="n">
-        <v>948</v>
+        <v>3223</v>
       </c>
       <c r="I95" t="b">
         <v>0</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>blasphemous, bloodborne, broodseeker, dark souls, elden ring, eredrim, h3llcreator, hadern, lady maria, lords of the fallen, malenia, mortal shell, mortal shell ii, proxima, tiel</t>
+          <t>3d print, 3mf, decor, decor master, decormaster, gift, multipart, no ams, toy</t>
         </is>
       </c>
       <c r="K95" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L95" t="n">
         <v>11.28571428571429</v>
       </c>
       <c r="M95" t="n">
-        <v>2780.8</v>
+        <v>625.6799999999999</v>
       </c>
       <c r="N95" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.04902264970524356</v>
       </c>
       <c r="O95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P95" t="b">
         <v>0</v>
@@ -10076,12 +10076,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>pin head Fan art (no ams-multiparts/3mf)</t>
+          <t>Proxima the Broodseeker</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:5055346</t>
+          <t>https://cults3d.com/:5079132</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -10090,42 +10090,42 @@
         </is>
       </c>
       <c r="D96" s="1" t="n">
-        <v>46308.81805555556</v>
+        <v>46313.49111111111</v>
       </c>
       <c r="E96" t="n">
-        <v>3.96</v>
+        <v>17.6</v>
       </c>
       <c r="F96" t="n">
         <v>158</v>
       </c>
       <c r="G96" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="H96" t="n">
-        <v>3223</v>
+        <v>949</v>
       </c>
       <c r="I96" t="b">
         <v>0</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>3d print, 3mf, decor, decor master, decormaster, gift, multipart, no ams, toy</t>
+          <t>blasphemous, bloodborne, broodseeker, dark souls, elden ring, eredrim, h3llcreator, hadern, lady maria, lords of the fallen, malenia, mortal shell, mortal shell ii, proxima, tiel</t>
         </is>
       </c>
       <c r="K96" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L96" t="n">
         <v>11.28571428571429</v>
       </c>
       <c r="M96" t="n">
-        <v>625.6799999999999</v>
+        <v>2780.8</v>
       </c>
       <c r="N96" t="n">
-        <v>0.04902264970524356</v>
+        <v>0.166491043203372</v>
       </c>
       <c r="O96" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P96" t="b">
         <v>0</v>
@@ -19174,12 +19174,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Spider Demon P2  (Head-Swap) by E.S Monster</t>
+          <t>ONI P2 (Head-Swap) by E.S Monster</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:4780086</t>
+          <t>https://cults3d.com/:4780060</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -19188,7 +19188,7 @@
         </is>
       </c>
       <c r="D253" s="1" t="n">
-        <v>46248.29128472223</v>
+        <v>46248.28496527778</v>
       </c>
       <c r="E253" t="n">
         <v>20</v>
@@ -19197,17 +19197,17 @@
         <v>237</v>
       </c>
       <c r="G253" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H253" t="n">
-        <v>749</v>
+        <v>657</v>
       </c>
       <c r="I253" t="b">
         <v>0</v>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>3d model, character, fanart, female, myth-inspired, sculpt, spider demon, stl</t>
+          <t>3d model, character, fanart, female, myth-inspired, oni, sculpt, stl</t>
         </is>
       </c>
       <c r="K253" t="n">
@@ -19220,10 +19220,10 @@
         <v>4740</v>
       </c>
       <c r="N253" t="n">
-        <v>0.3164218958611482</v>
+        <v>0.3607305936073059</v>
       </c>
       <c r="O253" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P253" t="b">
         <v>0</v>
@@ -19232,12 +19232,12 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>ONI P2 (Head-Swap) by E.S Monster</t>
+          <t>Spider Demon P2  (Head-Swap) by E.S Monster</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>https://cults3d.com/:4780060</t>
+          <t>https://cults3d.com/:4780086</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -19246,7 +19246,7 @@
         </is>
       </c>
       <c r="D254" s="1" t="n">
-        <v>46248.28496527778</v>
+        <v>46248.29128472223</v>
       </c>
       <c r="E254" t="n">
         <v>20</v>
@@ -19255,17 +19255,17 @@
         <v>237</v>
       </c>
       <c r="G254" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H254" t="n">
-        <v>657</v>
+        <v>749</v>
       </c>
       <c r="I254" t="b">
         <v>0</v>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>3d model, character, fanart, female, myth-inspired, oni, sculpt, stl</t>
+          <t>3d model, character, fanart, female, myth-inspired, sculpt, spider demon, stl</t>
         </is>
       </c>
       <c r="K254" t="n">
@@ -19278,10 +19278,10 @@
         <v>4740</v>
       </c>
       <c r="N254" t="n">
-        <v>0.3607305936073059</v>
+        <v>0.3164218958611482</v>
       </c>
       <c r="O254" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P254" t="b">
         <v>0</v>

</xml_diff>